<commit_message>
Add Parça Sayısı, Astar Durumu and Kalınlık columns to the added categories
Trendyol next asked for a Parça Sayısı column. Product pages in these
categories also use Astar Durumu (ceket) and Kalınlık (kazak), so add
all three at once; both two-piece sets get Parça Sayısı 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJxz6TxayURknP2UowWRAx
</commit_message>
<xml_diff>
--- a/minah-tekstil/trendyol/minah-trendyol-dosya-2.xlsx
+++ b/minah-tekstil/trendyol/minah-trendyol-dosya-2.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7117" uniqueCount="3467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7140" uniqueCount="3470">
   <si>
     <t>Barkod</t>
   </si>
@@ -10254,6 +10254,15 @@
   </si>
   <si>
     <t>Bu alanda "Hızlı Teslimat" ve "Bugün Kargoda" değişkenlerini ekleyebilirsiniz.</t>
+  </si>
+  <si>
+    <t>Parça Sayısı</t>
+  </si>
+  <si>
+    <t>Astar Durumu</t>
+  </si>
+  <si>
+    <t>Kalınlık</t>
   </si>
   <si>
     <t>MNH-POLO-TRIKO-KAZAK-TURUNCU-STD</t>
@@ -40198,7 +40207,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV13"/>
+  <dimension ref="A1:BY13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -40441,16 +40450,25 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3326</v>
+        <v>3329</v>
       </c>
       <c r="B2" t="s">
-        <v>3327</v>
+        <v>3330</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
         <v>360</v>
@@ -40459,10 +40477,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3329</v>
+        <v>3332</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3330</v>
+        <v>3333</v>
       </c>
       <c r="H2" s="38">
         <v>950</v>
@@ -40474,7 +40492,7 @@
         <v>5</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3326</v>
+        <v>3329</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -40527,13 +40545,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>3334</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3330</v>
+      </c>
+      <c r="C3" t="s">
         <v>3331</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3327</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3328</v>
       </c>
       <c r="D3" t="s">
         <v>360</v>
@@ -40545,7 +40563,7 @@
         <v>87</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3332</v>
+        <v>3335</v>
       </c>
       <c r="H3" s="38">
         <v>950</v>
@@ -40557,7 +40575,7 @@
         <v>5</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3331</v>
+        <v>3334</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -40590,7 +40608,7 @@
         <v>830</v>
       </c>
       <c r="AZ3" t="s">
-        <v>3333</v>
+        <v>3336</v>
       </c>
       <c r="BC3" t="s">
         <v>164</v>
@@ -40610,13 +40628,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3334</v>
+        <v>3337</v>
       </c>
       <c r="B4" t="s">
-        <v>3327</v>
+        <v>3330</v>
       </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
         <v>360</v>
@@ -40628,7 +40646,7 @@
         <v>97</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3335</v>
+        <v>3338</v>
       </c>
       <c r="H4" s="38">
         <v>950</v>
@@ -40640,7 +40658,7 @@
         <v>5</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3334</v>
+        <v>3337</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -40670,7 +40688,7 @@
         <v>830</v>
       </c>
       <c r="AZ4" t="s">
-        <v>3336</v>
+        <v>3339</v>
       </c>
       <c r="BC4" t="s">
         <v>164</v>
@@ -40690,13 +40708,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3337</v>
+        <v>3340</v>
       </c>
       <c r="B5" t="s">
-        <v>3327</v>
+        <v>3330</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
         <v>360</v>
@@ -40705,10 +40723,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3338</v>
+        <v>3341</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3339</v>
+        <v>3342</v>
       </c>
       <c r="H5" s="38">
         <v>950</v>
@@ -40720,7 +40738,7 @@
         <v>5</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3337</v>
+        <v>3340</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -40753,7 +40771,7 @@
         <v>830</v>
       </c>
       <c r="AZ5" t="s">
-        <v>3340</v>
+        <v>3343</v>
       </c>
       <c r="BC5" t="s">
         <v>164</v>
@@ -40773,13 +40791,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3341</v>
+        <v>3344</v>
       </c>
       <c r="B6" t="s">
-        <v>3342</v>
+        <v>3345</v>
       </c>
       <c r="C6" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D6" t="s">
         <v>360</v>
@@ -40788,10 +40806,10 @@
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3343</v>
+        <v>3346</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3344</v>
+        <v>3347</v>
       </c>
       <c r="H6" s="38">
         <v>800</v>
@@ -40803,7 +40821,7 @@
         <v>5</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3341</v>
+        <v>3344</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -40856,13 +40874,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>3348</v>
+      </c>
+      <c r="B7" t="s">
         <v>3345</v>
       </c>
-      <c r="B7" t="s">
-        <v>3342</v>
-      </c>
       <c r="C7" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D7" t="s">
         <v>360</v>
@@ -40871,10 +40889,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3346</v>
+        <v>3349</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3347</v>
+        <v>3350</v>
       </c>
       <c r="H7" s="38">
         <v>800</v>
@@ -40886,7 +40904,7 @@
         <v>5</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3345</v>
+        <v>3348</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -40936,13 +40954,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3348</v>
+        <v>3351</v>
       </c>
       <c r="B8" t="s">
-        <v>3342</v>
+        <v>3345</v>
       </c>
       <c r="C8" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D8" t="s">
         <v>360</v>
@@ -40951,10 +40969,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3349</v>
+        <v>3352</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3350</v>
+        <v>3353</v>
       </c>
       <c r="H8" s="38">
         <v>800</v>
@@ -40966,7 +40984,7 @@
         <v>5</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3348</v>
+        <v>3351</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -41019,13 +41037,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3351</v>
+        <v>3354</v>
       </c>
       <c r="B9" t="s">
-        <v>3352</v>
+        <v>3355</v>
       </c>
       <c r="C9" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D9" t="s">
         <v>360</v>
@@ -41034,10 +41052,10 @@
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3353</v>
+        <v>3356</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3354</v>
+        <v>3357</v>
       </c>
       <c r="H9" s="38">
         <v>1040</v>
@@ -41049,7 +41067,7 @@
         <v>20</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3351</v>
+        <v>3354</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -41099,13 +41117,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>3358</v>
+      </c>
+      <c r="B10" t="s">
         <v>3355</v>
       </c>
-      <c r="B10" t="s">
-        <v>3352</v>
-      </c>
       <c r="C10" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D10" t="s">
         <v>360</v>
@@ -41114,10 +41132,10 @@
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3356</v>
+        <v>3359</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3357</v>
+        <v>3360</v>
       </c>
       <c r="H10" s="38">
         <v>1040</v>
@@ -41129,7 +41147,7 @@
         <v>20</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3355</v>
+        <v>3358</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -41179,13 +41197,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3358</v>
+        <v>3361</v>
       </c>
       <c r="B11" t="s">
-        <v>3359</v>
+        <v>3362</v>
       </c>
       <c r="C11" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D11" t="s">
         <v>360</v>
@@ -41194,10 +41212,10 @@
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3360</v>
+        <v>3363</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3361</v>
+        <v>3364</v>
       </c>
       <c r="H11" s="38">
         <v>900</v>
@@ -41209,7 +41227,7 @@
         <v>5</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3358</v>
+        <v>3361</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -41242,7 +41260,7 @@
         <v>830</v>
       </c>
       <c r="AZ11" t="s">
-        <v>3362</v>
+        <v>3365</v>
       </c>
       <c r="BC11" t="s">
         <v>164</v>
@@ -41262,13 +41280,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3363</v>
+        <v>3366</v>
       </c>
       <c r="B12" t="s">
-        <v>3359</v>
+        <v>3362</v>
       </c>
       <c r="C12" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D12" t="s">
         <v>360</v>
@@ -41277,10 +41295,10 @@
         <v>70</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>3364</v>
+        <v>3367</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3365</v>
+        <v>3368</v>
       </c>
       <c r="H12" s="38">
         <v>900</v>
@@ -41292,7 +41310,7 @@
         <v>5</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3363</v>
+        <v>3366</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -41325,7 +41343,7 @@
         <v>830</v>
       </c>
       <c r="AZ12" t="s">
-        <v>3366</v>
+        <v>3369</v>
       </c>
       <c r="BC12" t="s">
         <v>164</v>
@@ -41345,13 +41363,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3367</v>
+        <v>3370</v>
       </c>
       <c r="B13" t="s">
-        <v>3359</v>
+        <v>3362</v>
       </c>
       <c r="C13" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D13" t="s">
         <v>360</v>
@@ -41360,10 +41378,10 @@
         <v>70</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>3368</v>
+        <v>3371</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3369</v>
+        <v>3372</v>
       </c>
       <c r="H13" s="38">
         <v>900</v>
@@ -41375,7 +41393,7 @@
         <v>5</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3367</v>
+        <v>3370</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -41405,7 +41423,7 @@
         <v>830</v>
       </c>
       <c r="AZ13" t="s">
-        <v>3370</v>
+        <v>3373</v>
       </c>
       <c r="BC13" t="s">
         <v>164</v>
@@ -43849,7 +43867,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV15"/>
+  <dimension ref="A1:BY15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -44092,16 +44110,25 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3371</v>
+        <v>3374</v>
       </c>
       <c r="B2" t="s">
-        <v>3372</v>
+        <v>3375</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
         <v>357</v>
@@ -44110,10 +44137,10 @@
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3373</v>
+        <v>3376</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3374</v>
+        <v>3377</v>
       </c>
       <c r="H2" s="38">
         <v>850</v>
@@ -44125,7 +44152,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3371</v>
+        <v>3374</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -44178,13 +44205,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>3378</v>
+      </c>
+      <c r="B3" t="s">
         <v>3375</v>
       </c>
-      <c r="B3" t="s">
-        <v>3372</v>
-      </c>
       <c r="C3" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D3" t="s">
         <v>357</v>
@@ -44193,10 +44220,10 @@
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3373</v>
+        <v>3376</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3374</v>
+        <v>3377</v>
       </c>
       <c r="H3" s="38">
         <v>850</v>
@@ -44208,7 +44235,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3375</v>
+        <v>3378</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -44261,13 +44288,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3376</v>
+        <v>3379</v>
       </c>
       <c r="B4" t="s">
-        <v>3372</v>
+        <v>3375</v>
       </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
         <v>357</v>
@@ -44276,10 +44303,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3373</v>
+        <v>3376</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3374</v>
+        <v>3377</v>
       </c>
       <c r="H4" s="38">
         <v>850</v>
@@ -44291,7 +44318,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3376</v>
+        <v>3379</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -44344,13 +44371,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3377</v>
+        <v>3380</v>
       </c>
       <c r="B5" t="s">
-        <v>3372</v>
+        <v>3375</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
         <v>357</v>
@@ -44359,10 +44386,10 @@
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3373</v>
+        <v>3376</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3374</v>
+        <v>3377</v>
       </c>
       <c r="H5" s="38">
         <v>850</v>
@@ -44374,7 +44401,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3377</v>
+        <v>3380</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -44427,13 +44454,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3378</v>
+        <v>3381</v>
       </c>
       <c r="B6" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C6" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D6" t="s">
         <v>357</v>
@@ -44442,10 +44469,10 @@
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3380</v>
+        <v>3383</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3381</v>
+        <v>3384</v>
       </c>
       <c r="H6" s="38">
         <v>1050</v>
@@ -44457,7 +44484,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3378</v>
+        <v>3381</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -44507,13 +44534,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>3385</v>
+      </c>
+      <c r="B7" t="s">
         <v>3382</v>
       </c>
-      <c r="B7" t="s">
-        <v>3379</v>
-      </c>
       <c r="C7" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D7" t="s">
         <v>357</v>
@@ -44522,10 +44549,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3380</v>
+        <v>3383</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3381</v>
+        <v>3384</v>
       </c>
       <c r="H7" s="38">
         <v>1050</v>
@@ -44537,7 +44564,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3382</v>
+        <v>3385</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -44587,13 +44614,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3383</v>
+        <v>3386</v>
       </c>
       <c r="B8" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C8" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D8" t="s">
         <v>357</v>
@@ -44602,10 +44629,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3380</v>
+        <v>3383</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3381</v>
+        <v>3384</v>
       </c>
       <c r="H8" s="38">
         <v>1050</v>
@@ -44617,7 +44644,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3383</v>
+        <v>3386</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -44667,13 +44694,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3384</v>
+        <v>3387</v>
       </c>
       <c r="B9" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C9" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D9" t="s">
         <v>357</v>
@@ -44682,10 +44709,10 @@
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3380</v>
+        <v>3383</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3381</v>
+        <v>3384</v>
       </c>
       <c r="H9" s="38">
         <v>1050</v>
@@ -44697,7 +44724,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3384</v>
+        <v>3387</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -44747,13 +44774,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3385</v>
+        <v>3388</v>
       </c>
       <c r="B10" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C10" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D10" t="s">
         <v>357</v>
@@ -44762,10 +44789,10 @@
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3380</v>
+        <v>3383</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3381</v>
+        <v>3384</v>
       </c>
       <c r="H10" s="38">
         <v>1050</v>
@@ -44777,7 +44804,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3385</v>
+        <v>3388</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -44827,13 +44854,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3386</v>
+        <v>3389</v>
       </c>
       <c r="B11" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C11" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D11" t="s">
         <v>357</v>
@@ -44842,10 +44869,10 @@
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3387</v>
+        <v>3390</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3388</v>
+        <v>3391</v>
       </c>
       <c r="H11" s="38">
         <v>1050</v>
@@ -44857,7 +44884,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3386</v>
+        <v>3389</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -44907,13 +44934,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3389</v>
+        <v>3392</v>
       </c>
       <c r="B12" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C12" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D12" t="s">
         <v>357</v>
@@ -44922,10 +44949,10 @@
         <v>70</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>3387</v>
+        <v>3390</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3388</v>
+        <v>3391</v>
       </c>
       <c r="H12" s="38">
         <v>1050</v>
@@ -44937,7 +44964,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3389</v>
+        <v>3392</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -44987,13 +45014,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3390</v>
+        <v>3393</v>
       </c>
       <c r="B13" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C13" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D13" t="s">
         <v>357</v>
@@ -45002,10 +45029,10 @@
         <v>70</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>3387</v>
+        <v>3390</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3388</v>
+        <v>3391</v>
       </c>
       <c r="H13" s="38">
         <v>1050</v>
@@ -45017,7 +45044,7 @@
         <v>1</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3390</v>
+        <v>3393</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -45067,13 +45094,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>3391</v>
+        <v>3394</v>
       </c>
       <c r="B14" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C14" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D14" t="s">
         <v>357</v>
@@ -45082,10 +45109,10 @@
         <v>70</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>3387</v>
+        <v>3390</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>3388</v>
+        <v>3391</v>
       </c>
       <c r="H14" s="38">
         <v>1050</v>
@@ -45097,7 +45124,7 @@
         <v>1</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>3391</v>
+        <v>3394</v>
       </c>
       <c r="L14" s="39">
         <v>10</v>
@@ -45147,13 +45174,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>3392</v>
+        <v>3395</v>
       </c>
       <c r="B15" t="s">
-        <v>3379</v>
+        <v>3382</v>
       </c>
       <c r="C15" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D15" t="s">
         <v>357</v>
@@ -45162,10 +45189,10 @@
         <v>70</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>3387</v>
+        <v>3390</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>3388</v>
+        <v>3391</v>
       </c>
       <c r="H15" s="38">
         <v>1050</v>
@@ -45177,7 +45204,7 @@
         <v>1</v>
       </c>
       <c r="K15" s="39" t="s">
-        <v>3392</v>
+        <v>3395</v>
       </c>
       <c r="L15" s="39">
         <v>10</v>
@@ -47651,7 +47678,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV16"/>
+  <dimension ref="A1:BY16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -47894,16 +47921,25 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3393</v>
+        <v>3396</v>
       </c>
       <c r="B2" t="s">
-        <v>3394</v>
+        <v>3397</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
         <v>333</v>
@@ -47915,7 +47951,7 @@
         <v>183</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3395</v>
+        <v>3398</v>
       </c>
       <c r="H2" s="38">
         <v>799</v>
@@ -47927,7 +47963,7 @@
         <v>2</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3393</v>
+        <v>3396</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -47980,13 +48016,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3396</v>
+        <v>3399</v>
       </c>
       <c r="B3" t="s">
-        <v>3394</v>
+        <v>3397</v>
       </c>
       <c r="C3" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D3" t="s">
         <v>333</v>
@@ -47998,7 +48034,7 @@
         <v>183</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3395</v>
+        <v>3398</v>
       </c>
       <c r="H3" s="38">
         <v>799</v>
@@ -48010,7 +48046,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3396</v>
+        <v>3399</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -48063,13 +48099,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>3400</v>
+      </c>
+      <c r="B4" t="s">
         <v>3397</v>
       </c>
-      <c r="B4" t="s">
-        <v>3394</v>
-      </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
         <v>333</v>
@@ -48081,7 +48117,7 @@
         <v>183</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3395</v>
+        <v>3398</v>
       </c>
       <c r="H4" s="38">
         <v>799</v>
@@ -48093,7 +48129,7 @@
         <v>2</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3397</v>
+        <v>3400</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -48146,13 +48182,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3398</v>
+        <v>3401</v>
       </c>
       <c r="B5" t="s">
-        <v>3394</v>
+        <v>3397</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
         <v>333</v>
@@ -48164,7 +48200,7 @@
         <v>183</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3395</v>
+        <v>3398</v>
       </c>
       <c r="H5" s="38">
         <v>799</v>
@@ -48176,7 +48212,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3398</v>
+        <v>3401</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -48229,13 +48265,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3399</v>
+        <v>3402</v>
       </c>
       <c r="B6" t="s">
-        <v>3394</v>
+        <v>3397</v>
       </c>
       <c r="C6" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D6" t="s">
         <v>333</v>
@@ -48247,7 +48283,7 @@
         <v>183</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3395</v>
+        <v>3398</v>
       </c>
       <c r="H6" s="38">
         <v>799</v>
@@ -48259,7 +48295,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3399</v>
+        <v>3402</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -48312,13 +48348,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3400</v>
+        <v>3403</v>
       </c>
       <c r="B7" t="s">
-        <v>3401</v>
+        <v>3404</v>
       </c>
       <c r="C7" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D7" t="s">
         <v>333</v>
@@ -48327,10 +48363,10 @@
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3402</v>
+        <v>3405</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="H7" s="38">
         <v>785</v>
@@ -48342,7 +48378,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3400</v>
+        <v>3403</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -48395,13 +48431,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>3407</v>
+      </c>
+      <c r="B8" t="s">
         <v>3404</v>
       </c>
-      <c r="B8" t="s">
-        <v>3401</v>
-      </c>
       <c r="C8" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D8" t="s">
         <v>333</v>
@@ -48410,10 +48446,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3402</v>
+        <v>3405</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="H8" s="38">
         <v>785</v>
@@ -48425,7 +48461,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3404</v>
+        <v>3407</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -48478,13 +48514,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3405</v>
+        <v>3408</v>
       </c>
       <c r="B9" t="s">
-        <v>3401</v>
+        <v>3404</v>
       </c>
       <c r="C9" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D9" t="s">
         <v>333</v>
@@ -48493,10 +48529,10 @@
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3402</v>
+        <v>3405</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="H9" s="38">
         <v>785</v>
@@ -48508,7 +48544,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3405</v>
+        <v>3408</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -48561,13 +48597,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3406</v>
+        <v>3409</v>
       </c>
       <c r="B10" t="s">
-        <v>3401</v>
+        <v>3404</v>
       </c>
       <c r="C10" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D10" t="s">
         <v>333</v>
@@ -48576,10 +48612,10 @@
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3402</v>
+        <v>3405</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="H10" s="38">
         <v>785</v>
@@ -48591,7 +48627,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3406</v>
+        <v>3409</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -48644,13 +48680,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3407</v>
+        <v>3410</v>
       </c>
       <c r="B11" t="s">
-        <v>3401</v>
+        <v>3404</v>
       </c>
       <c r="C11" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D11" t="s">
         <v>333</v>
@@ -48659,10 +48695,10 @@
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3402</v>
+        <v>3405</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="H11" s="38">
         <v>785</v>
@@ -48674,7 +48710,7 @@
         <v>2</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3407</v>
+        <v>3410</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -48727,13 +48763,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3408</v>
+        <v>3411</v>
       </c>
       <c r="B12" t="s">
-        <v>3409</v>
+        <v>3412</v>
       </c>
       <c r="C12" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D12" t="s">
         <v>333</v>
@@ -48745,7 +48781,7 @@
         <v>265</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3410</v>
+        <v>3413</v>
       </c>
       <c r="H12" s="38">
         <v>800</v>
@@ -48757,7 +48793,7 @@
         <v>2</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3408</v>
+        <v>3411</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -48807,13 +48843,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3411</v>
+        <v>3414</v>
       </c>
       <c r="B13" t="s">
-        <v>3409</v>
+        <v>3412</v>
       </c>
       <c r="C13" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D13" t="s">
         <v>333</v>
@@ -48825,7 +48861,7 @@
         <v>265</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3410</v>
+        <v>3413</v>
       </c>
       <c r="H13" s="38">
         <v>800</v>
@@ -48837,7 +48873,7 @@
         <v>2</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3411</v>
+        <v>3414</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -48887,13 +48923,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>3415</v>
+      </c>
+      <c r="B14" t="s">
         <v>3412</v>
       </c>
-      <c r="B14" t="s">
-        <v>3409</v>
-      </c>
       <c r="C14" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D14" t="s">
         <v>333</v>
@@ -48905,7 +48941,7 @@
         <v>265</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>3410</v>
+        <v>3413</v>
       </c>
       <c r="H14" s="38">
         <v>800</v>
@@ -48917,7 +48953,7 @@
         <v>2</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>3412</v>
+        <v>3415</v>
       </c>
       <c r="L14" s="39">
         <v>10</v>
@@ -48967,13 +49003,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>3413</v>
+        <v>3416</v>
       </c>
       <c r="B15" t="s">
-        <v>3409</v>
+        <v>3412</v>
       </c>
       <c r="C15" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D15" t="s">
         <v>333</v>
@@ -48985,7 +49021,7 @@
         <v>265</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>3410</v>
+        <v>3413</v>
       </c>
       <c r="H15" s="38">
         <v>800</v>
@@ -48997,7 +49033,7 @@
         <v>2</v>
       </c>
       <c r="K15" s="39" t="s">
-        <v>3413</v>
+        <v>3416</v>
       </c>
       <c r="L15" s="39">
         <v>10</v>
@@ -49047,13 +49083,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>3414</v>
+        <v>3417</v>
       </c>
       <c r="B16" t="s">
-        <v>3409</v>
+        <v>3412</v>
       </c>
       <c r="C16" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D16" t="s">
         <v>333</v>
@@ -49065,7 +49101,7 @@
         <v>265</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>3410</v>
+        <v>3413</v>
       </c>
       <c r="H16" s="38">
         <v>800</v>
@@ -49077,7 +49113,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="39" t="s">
-        <v>3414</v>
+        <v>3417</v>
       </c>
       <c r="L16" s="39">
         <v>10</v>
@@ -51551,7 +51587,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV19"/>
+  <dimension ref="A1:BY19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -51794,28 +51830,37 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3415</v>
+        <v>3418</v>
       </c>
       <c r="B2" t="s">
-        <v>3416</v>
+        <v>3419</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E2" t="s">
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H2" s="38">
         <v>500</v>
@@ -51827,7 +51872,7 @@
         <v>2</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3415</v>
+        <v>3418</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -51877,25 +51922,25 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>3423</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3419</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3331</v>
+      </c>
+      <c r="D3" t="s">
         <v>3420</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3416</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3328</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3417</v>
       </c>
       <c r="E3" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H3" s="38">
         <v>500</v>
@@ -51907,7 +51952,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3420</v>
+        <v>3423</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -51957,25 +52002,25 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3421</v>
+        <v>3424</v>
       </c>
       <c r="B4" t="s">
-        <v>3416</v>
+        <v>3419</v>
       </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E4" t="s">
         <v>70</v>
       </c>
       <c r="F4" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H4" s="38">
         <v>500</v>
@@ -51987,7 +52032,7 @@
         <v>2</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3421</v>
+        <v>3424</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -52037,25 +52082,25 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3422</v>
+        <v>3425</v>
       </c>
       <c r="B5" t="s">
-        <v>3416</v>
+        <v>3419</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E5" t="s">
         <v>70</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H5" s="38">
         <v>500</v>
@@ -52067,7 +52112,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3422</v>
+        <v>3425</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -52117,25 +52162,25 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3423</v>
+        <v>3426</v>
       </c>
       <c r="B6" t="s">
-        <v>3416</v>
+        <v>3419</v>
       </c>
       <c r="C6" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D6" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E6" t="s">
         <v>70</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H6" s="38">
         <v>500</v>
@@ -52147,7 +52192,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3423</v>
+        <v>3426</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -52197,25 +52242,25 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3424</v>
+        <v>3427</v>
       </c>
       <c r="B7" t="s">
-        <v>3416</v>
+        <v>3419</v>
       </c>
       <c r="C7" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D7" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E7" t="s">
         <v>70</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>3418</v>
+        <v>3421</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3419</v>
+        <v>3422</v>
       </c>
       <c r="H7" s="38">
         <v>500</v>
@@ -52227,7 +52272,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3424</v>
+        <v>3427</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -52277,25 +52322,25 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3425</v>
+        <v>3428</v>
       </c>
       <c r="B8" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C8" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D8" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E8" t="s">
         <v>70</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H8" s="38">
         <v>500</v>
@@ -52307,7 +52352,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3425</v>
+        <v>3428</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -52351,25 +52396,25 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>3432</v>
+      </c>
+      <c r="B9" t="s">
         <v>3429</v>
       </c>
-      <c r="B9" t="s">
-        <v>3426</v>
-      </c>
       <c r="C9" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D9" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E9" t="s">
         <v>70</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H9" s="38">
         <v>500</v>
@@ -52381,7 +52426,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3429</v>
+        <v>3432</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -52425,25 +52470,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>3430</v>
+        <v>3433</v>
       </c>
       <c r="B10" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C10" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D10" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E10" t="s">
         <v>70</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H10" s="38">
         <v>500</v>
@@ -52455,7 +52500,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="39" t="s">
-        <v>3430</v>
+        <v>3433</v>
       </c>
       <c r="L10" s="39">
         <v>10</v>
@@ -52499,25 +52544,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3431</v>
+        <v>3434</v>
       </c>
       <c r="B11" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C11" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D11" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E11" t="s">
         <v>70</v>
       </c>
       <c r="F11" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H11" s="38">
         <v>500</v>
@@ -52529,7 +52574,7 @@
         <v>2</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>3431</v>
+        <v>3434</v>
       </c>
       <c r="L11" s="39">
         <v>10</v>
@@ -52573,25 +52618,25 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3432</v>
+        <v>3435</v>
       </c>
       <c r="B12" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C12" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D12" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E12" t="s">
         <v>70</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H12" s="38">
         <v>500</v>
@@ -52603,7 +52648,7 @@
         <v>2</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>3432</v>
+        <v>3435</v>
       </c>
       <c r="L12" s="39">
         <v>10</v>
@@ -52647,25 +52692,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>3433</v>
+        <v>3436</v>
       </c>
       <c r="B13" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C13" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D13" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E13" t="s">
         <v>70</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>3427</v>
+        <v>3430</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>3428</v>
+        <v>3431</v>
       </c>
       <c r="H13" s="38">
         <v>500</v>
@@ -52677,7 +52722,7 @@
         <v>2</v>
       </c>
       <c r="K13" s="39" t="s">
-        <v>3433</v>
+        <v>3436</v>
       </c>
       <c r="L13" s="39">
         <v>10</v>
@@ -52721,25 +52766,25 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>3434</v>
+        <v>3437</v>
       </c>
       <c r="B14" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C14" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D14" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E14" t="s">
         <v>70</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H14" s="38">
         <v>550</v>
@@ -52751,7 +52796,7 @@
         <v>2</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>3434</v>
+        <v>3437</v>
       </c>
       <c r="L14" s="39">
         <v>10</v>
@@ -52801,25 +52846,25 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>3437</v>
+        <v>3440</v>
       </c>
       <c r="B15" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C15" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D15" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E15" t="s">
         <v>70</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H15" s="38">
         <v>550</v>
@@ -52831,7 +52876,7 @@
         <v>2</v>
       </c>
       <c r="K15" s="39" t="s">
-        <v>3437</v>
+        <v>3440</v>
       </c>
       <c r="L15" s="39">
         <v>10</v>
@@ -52881,25 +52926,25 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>3438</v>
+        <v>3441</v>
       </c>
       <c r="B16" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C16" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D16" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E16" t="s">
         <v>70</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H16" s="38">
         <v>550</v>
@@ -52911,7 +52956,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="39" t="s">
-        <v>3438</v>
+        <v>3441</v>
       </c>
       <c r="L16" s="39">
         <v>10</v>
@@ -52961,25 +53006,25 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>3439</v>
+        <v>3442</v>
       </c>
       <c r="B17" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C17" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D17" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E17" t="s">
         <v>70</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G17" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H17" s="38">
         <v>550</v>
@@ -52991,7 +53036,7 @@
         <v>2</v>
       </c>
       <c r="K17" s="39" t="s">
-        <v>3439</v>
+        <v>3442</v>
       </c>
       <c r="L17" s="39">
         <v>10</v>
@@ -53041,25 +53086,25 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>3440</v>
+        <v>3443</v>
       </c>
       <c r="B18" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C18" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D18" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E18" t="s">
         <v>70</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H18" s="38">
         <v>550</v>
@@ -53071,7 +53116,7 @@
         <v>2</v>
       </c>
       <c r="K18" s="39" t="s">
-        <v>3440</v>
+        <v>3443</v>
       </c>
       <c r="L18" s="39">
         <v>10</v>
@@ -53121,25 +53166,25 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>3441</v>
+        <v>3444</v>
       </c>
       <c r="B19" t="s">
-        <v>3426</v>
+        <v>3429</v>
       </c>
       <c r="C19" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D19" t="s">
-        <v>3417</v>
+        <v>3420</v>
       </c>
       <c r="E19" t="s">
         <v>70</v>
       </c>
       <c r="F19" s="35" t="s">
-        <v>3435</v>
+        <v>3438</v>
       </c>
       <c r="G19" s="35" t="s">
-        <v>3436</v>
+        <v>3439</v>
       </c>
       <c r="H19" s="38">
         <v>550</v>
@@ -53151,7 +53196,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="39" t="s">
-        <v>3441</v>
+        <v>3444</v>
       </c>
       <c r="L19" s="39">
         <v>10</v>
@@ -55625,7 +55670,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV5"/>
+  <dimension ref="A1:BY5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -55868,16 +55913,25 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3442</v>
+        <v>3445</v>
       </c>
       <c r="B2" t="s">
-        <v>3443</v>
+        <v>3446</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
         <v>375</v>
@@ -55889,7 +55943,7 @@
         <v>361</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3444</v>
+        <v>3447</v>
       </c>
       <c r="H2" s="38">
         <v>250</v>
@@ -55901,7 +55955,7 @@
         <v>8</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3442</v>
+        <v>3445</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -55951,13 +56005,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3445</v>
+        <v>3448</v>
       </c>
       <c r="B3" t="s">
-        <v>3443</v>
+        <v>3446</v>
       </c>
       <c r="C3" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D3" t="s">
         <v>375</v>
@@ -55969,7 +56023,7 @@
         <v>361</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3444</v>
+        <v>3447</v>
       </c>
       <c r="H3" s="38">
         <v>250</v>
@@ -55981,7 +56035,7 @@
         <v>8</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3445</v>
+        <v>3448</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -56031,13 +56085,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>3449</v>
+      </c>
+      <c r="B4" t="s">
         <v>3446</v>
       </c>
-      <c r="B4" t="s">
-        <v>3443</v>
-      </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
         <v>375</v>
@@ -56049,7 +56103,7 @@
         <v>361</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3444</v>
+        <v>3447</v>
       </c>
       <c r="H4" s="38">
         <v>250</v>
@@ -56061,7 +56115,7 @@
         <v>8</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3446</v>
+        <v>3449</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -56111,13 +56165,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3447</v>
+        <v>3450</v>
       </c>
       <c r="B5" t="s">
-        <v>3443</v>
+        <v>3446</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
         <v>375</v>
@@ -56129,7 +56183,7 @@
         <v>361</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3444</v>
+        <v>3447</v>
       </c>
       <c r="H5" s="38">
         <v>250</v>
@@ -56141,7 +56195,7 @@
         <v>8</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3447</v>
+        <v>3450</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -58615,7 +58669,7 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV9"/>
+  <dimension ref="A1:BY9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -58858,16 +58912,25 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3448</v>
+        <v>3451</v>
       </c>
       <c r="B2" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
         <v>349</v>
@@ -58879,7 +58942,7 @@
         <v>520</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3450</v>
+        <v>3453</v>
       </c>
       <c r="H2" s="38">
         <v>1600</v>
@@ -58891,7 +58954,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3448</v>
+        <v>3451</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -58941,13 +59004,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3451</v>
+        <v>3454</v>
       </c>
       <c r="B3" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C3" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D3" t="s">
         <v>349</v>
@@ -58959,7 +59022,7 @@
         <v>520</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3450</v>
+        <v>3453</v>
       </c>
       <c r="H3" s="38">
         <v>1600</v>
@@ -58971,7 +59034,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3451</v>
+        <v>3454</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -59021,13 +59084,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>3455</v>
+      </c>
+      <c r="B4" t="s">
         <v>3452</v>
       </c>
-      <c r="B4" t="s">
-        <v>3449</v>
-      </c>
       <c r="C4" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D4" t="s">
         <v>349</v>
@@ -59039,7 +59102,7 @@
         <v>520</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>3450</v>
+        <v>3453</v>
       </c>
       <c r="H4" s="38">
         <v>1600</v>
@@ -59051,7 +59114,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="39" t="s">
-        <v>3452</v>
+        <v>3455</v>
       </c>
       <c r="L4" s="39">
         <v>10</v>
@@ -59101,13 +59164,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3453</v>
+        <v>3456</v>
       </c>
       <c r="B5" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C5" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D5" t="s">
         <v>349</v>
@@ -59119,7 +59182,7 @@
         <v>520</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>3450</v>
+        <v>3453</v>
       </c>
       <c r="H5" s="38">
         <v>1600</v>
@@ -59131,7 +59194,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>3453</v>
+        <v>3456</v>
       </c>
       <c r="L5" s="39">
         <v>10</v>
@@ -59181,13 +59244,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3454</v>
+        <v>3457</v>
       </c>
       <c r="B6" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C6" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D6" t="s">
         <v>349</v>
@@ -59199,7 +59262,7 @@
         <v>533</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>3455</v>
+        <v>3458</v>
       </c>
       <c r="H6" s="38">
         <v>1600</v>
@@ -59211,7 +59274,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>3454</v>
+        <v>3457</v>
       </c>
       <c r="L6" s="39">
         <v>10</v>
@@ -59264,13 +59327,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3456</v>
+        <v>3459</v>
       </c>
       <c r="B7" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C7" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D7" t="s">
         <v>349</v>
@@ -59282,7 +59345,7 @@
         <v>533</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>3455</v>
+        <v>3458</v>
       </c>
       <c r="H7" s="38">
         <v>1600</v>
@@ -59294,7 +59357,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>3456</v>
+        <v>3459</v>
       </c>
       <c r="L7" s="39">
         <v>10</v>
@@ -59347,13 +59410,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3457</v>
+        <v>3460</v>
       </c>
       <c r="B8" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C8" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D8" t="s">
         <v>349</v>
@@ -59365,7 +59428,7 @@
         <v>533</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>3455</v>
+        <v>3458</v>
       </c>
       <c r="H8" s="38">
         <v>1600</v>
@@ -59377,7 +59440,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="39" t="s">
-        <v>3457</v>
+        <v>3460</v>
       </c>
       <c r="L8" s="39">
         <v>10</v>
@@ -59430,13 +59493,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>3458</v>
+        <v>3461</v>
       </c>
       <c r="B9" t="s">
-        <v>3449</v>
+        <v>3452</v>
       </c>
       <c r="C9" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D9" t="s">
         <v>349</v>
@@ -59448,7 +59511,7 @@
         <v>533</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>3455</v>
+        <v>3458</v>
       </c>
       <c r="H9" s="38">
         <v>1600</v>
@@ -59460,7 +59523,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="39" t="s">
-        <v>3458</v>
+        <v>3461</v>
       </c>
       <c r="L9" s="39">
         <v>10</v>
@@ -61937,7 +62000,7 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV3"/>
+  <dimension ref="A1:BY3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -62180,28 +62243,37 @@
       <c r="BV1" s="41" t="s">
         <v>1846</v>
       </c>
+      <c r="BW1" s="41" t="s">
+        <v>3326</v>
+      </c>
+      <c r="BX1" s="41" t="s">
+        <v>3327</v>
+      </c>
+      <c r="BY1" s="41" t="s">
+        <v>3328</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3459</v>
+        <v>3462</v>
       </c>
       <c r="B2" t="s">
-        <v>3460</v>
+        <v>3463</v>
       </c>
       <c r="C2" t="s">
-        <v>3328</v>
+        <v>3331</v>
       </c>
       <c r="D2" t="s">
-        <v>3461</v>
+        <v>3464</v>
       </c>
       <c r="E2" t="s">
         <v>70</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>3462</v>
+        <v>3465</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>3463</v>
+        <v>3466</v>
       </c>
       <c r="H2" s="38">
         <v>1000</v>
@@ -62213,7 +62285,7 @@
         <v>5</v>
       </c>
       <c r="K2" s="39" t="s">
-        <v>3459</v>
+        <v>3462</v>
       </c>
       <c r="L2" s="39">
         <v>10</v>
@@ -62254,28 +62326,31 @@
       <c r="BL2" t="s">
         <v>164</v>
       </c>
+      <c r="BW2" t="s">
+        <v>678</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>3467</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3463</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3331</v>
+      </c>
+      <c r="D3" t="s">
         <v>3464</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3460</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3328</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3461</v>
       </c>
       <c r="E3" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>3465</v>
+        <v>3468</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>3466</v>
+        <v>3469</v>
       </c>
       <c r="H3" s="38">
         <v>1000</v>
@@ -62287,7 +62362,7 @@
         <v>5</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>3464</v>
+        <v>3467</v>
       </c>
       <c r="L3" s="39">
         <v>10</v>
@@ -62327,6 +62402,9 @@
       </c>
       <c r="BL3" t="s">
         <v>164</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>